<commit_message>
Fix Excel errors: replace all formulas with computed values
Root cause: openpyxl writes formulas without cached values, causing
errors in Excel Online and GitHub preview.

Fix: All formula cells (costs, margins, rolling mill, NCR cross-refs)
are now computed in Python and written as plain numbers. Zero formulas
remain in the output files.

Also regenerated both 23 Mar and 26 Mar outputs with correct values.

https://claude.ai/code/session_0134QcDJAg7cq3Eyj1JQx4hr
</commit_message>
<xml_diff>
--- a/output/2026-03-23/20260323_Costing TMT.xlsx
+++ b/output/2026-03-23/20260323_Costing TMT.xlsx
@@ -1923,20 +1923,17 @@
       <c r="E7" s="188" t="n">
         <v>26300</v>
       </c>
-      <c r="F7" s="189">
-        <f>E7*C7/100</f>
-        <v/>
+      <c r="F7" s="189" t="n">
+        <v>17884</v>
       </c>
       <c r="G7" s="190" t="n">
         <v>0.8</v>
       </c>
-      <c r="H7" s="189">
-        <f>F7/G7</f>
-        <v/>
-      </c>
-      <c r="I7" s="189">
-        <f>H7</f>
-        <v/>
+      <c r="H7" s="189" t="n">
+        <v>22355</v>
+      </c>
+      <c r="I7" s="189" t="n">
+        <v>22355</v>
       </c>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
@@ -1973,20 +1970,17 @@
       <c r="E8" s="188" t="n">
         <v>37300</v>
       </c>
-      <c r="F8" s="196">
-        <f>E8*C8/100</f>
-        <v/>
+      <c r="F8" s="196" t="n">
+        <v>4476</v>
       </c>
       <c r="G8" s="197" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="H8" s="196">
-        <f>F8/G8</f>
-        <v/>
-      </c>
-      <c r="I8" s="196">
-        <f>H8</f>
-        <v/>
+      <c r="H8" s="196" t="n">
+        <v>4761.7</v>
+      </c>
+      <c r="I8" s="196" t="n">
+        <v>4761.7</v>
       </c>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
@@ -2023,20 +2017,17 @@
       <c r="E9" s="188" t="n">
         <v>34900</v>
       </c>
-      <c r="F9" s="189">
-        <f>E9*C9/100</f>
-        <v/>
+      <c r="F9" s="189" t="n">
+        <v>3490</v>
       </c>
       <c r="G9" s="190" t="n">
         <v>0.96</v>
       </c>
-      <c r="H9" s="189">
-        <f>F9/G9</f>
-        <v/>
-      </c>
-      <c r="I9" s="189">
-        <f>H9</f>
-        <v/>
+      <c r="H9" s="189" t="n">
+        <v>3635.42</v>
+      </c>
+      <c r="I9" s="189" t="n">
+        <v>3635.42</v>
       </c>
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
@@ -2071,20 +2062,17 @@
       <c r="E10" s="188" t="n">
         <v>74.59999999999999</v>
       </c>
-      <c r="F10" s="196">
-        <f>E10*C10</f>
-        <v/>
+      <c r="F10" s="196" t="n">
+        <v>1044.4</v>
       </c>
       <c r="G10" s="197" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="196">
-        <f>F10/G10</f>
-        <v/>
-      </c>
-      <c r="I10" s="196">
-        <f>H10</f>
-        <v/>
+      <c r="H10" s="196" t="n">
+        <v>1044.4</v>
+      </c>
+      <c r="I10" s="196" t="n">
+        <v>1044.4</v>
       </c>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
@@ -2121,20 +2109,17 @@
       <c r="E11" s="188" t="n">
         <v>30200</v>
       </c>
-      <c r="F11" s="189">
-        <f>E11*C11/100</f>
-        <v/>
+      <c r="F11" s="189" t="n">
+        <v>3020</v>
       </c>
       <c r="G11" s="190" t="n">
         <v>0.84</v>
       </c>
-      <c r="H11" s="189">
-        <f>F11/G11</f>
-        <v/>
-      </c>
-      <c r="I11" s="189">
-        <f>H11</f>
-        <v/>
+      <c r="H11" s="189" t="n">
+        <v>3595.24</v>
+      </c>
+      <c r="I11" s="189" t="n">
+        <v>3595.24</v>
       </c>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
@@ -2165,15 +2150,13 @@
       <c r="E12" s="188" t="n">
         <v>6.5</v>
       </c>
-      <c r="F12" s="196">
-        <f>E12*C12</f>
-        <v/>
+      <c r="F12" s="196" t="n">
+        <v>4550</v>
       </c>
       <c r="G12" s="197" t="n"/>
       <c r="H12" s="200" t="n"/>
-      <c r="I12" s="196">
-        <f>E12*C12</f>
-        <v/>
+      <c r="I12" s="196" t="n">
+        <v>4550</v>
       </c>
       <c r="J12" s="5" t="n"/>
       <c r="K12" s="5" t="n"/>
@@ -2208,9 +2191,8 @@
       <c r="E13" s="188" t="n">
         <v>500</v>
       </c>
-      <c r="F13" s="189">
-        <f>E13*C13</f>
-        <v/>
+      <c r="F13" s="189" t="n">
+        <v>500</v>
       </c>
       <c r="G13" s="190" t="n"/>
       <c r="H13" s="202" t="n"/>
@@ -2250,9 +2232,8 @@
       <c r="E14" s="188" t="n">
         <v>550</v>
       </c>
-      <c r="F14" s="196">
-        <f>E14</f>
-        <v/>
+      <c r="F14" s="196" t="n">
+        <v>550</v>
       </c>
       <c r="G14" s="197" t="n"/>
       <c r="H14" s="200" t="n"/>
@@ -2287,9 +2268,8 @@
       <c r="F15" s="205" t="n"/>
       <c r="G15" s="205" t="n"/>
       <c r="H15" s="205" t="n"/>
-      <c r="I15" s="206">
-        <f>SUM(I7:I14)</f>
-        <v/>
+      <c r="I15" s="206" t="n">
+        <v>40991.76</v>
       </c>
       <c r="J15" s="12" t="n"/>
       <c r="K15" s="12" t="n"/>
@@ -2348,9 +2328,8 @@
       <c r="F17" s="205" t="n"/>
       <c r="G17" s="205" t="n"/>
       <c r="H17" s="205" t="n"/>
-      <c r="I17" s="206">
-        <f>I16-I15</f>
-        <v/>
+      <c r="I17" s="206" t="n">
+        <v>558.24</v>
       </c>
       <c r="J17" s="18" t="n"/>
       <c r="K17" s="18" t="n"/>
@@ -2481,9 +2460,8 @@
       <c r="C21" s="202" t="n"/>
       <c r="D21" s="202" t="n"/>
       <c r="E21" s="202" t="n"/>
-      <c r="F21" s="189">
-        <f>I15</f>
-        <v/>
+      <c r="F21" s="189" t="n">
+        <v>40991.76</v>
       </c>
       <c r="G21" s="141" t="n"/>
       <c r="H21" s="141" t="n"/>
@@ -2520,13 +2498,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="E22" s="196">
-        <f>I15</f>
-        <v/>
-      </c>
-      <c r="F22" s="196">
-        <f>E22*C22/100</f>
-        <v/>
+      <c r="E22" s="196" t="n">
+        <v>40991.76</v>
+      </c>
+      <c r="F22" s="196" t="n">
+        <v>327.93</v>
       </c>
       <c r="G22" s="140" t="n"/>
       <c r="H22" s="140" t="n"/>
@@ -2566,9 +2542,8 @@
       <c r="E23" s="189" t="n">
         <v>6.5</v>
       </c>
-      <c r="F23" s="189">
-        <f>E23*C23</f>
-        <v/>
+      <c r="F23" s="189" t="n">
+        <v>780</v>
       </c>
       <c r="G23" s="140" t="n"/>
       <c r="H23" s="140" t="n"/>
@@ -2608,9 +2583,8 @@
       <c r="E24" s="196" t="n">
         <v>400</v>
       </c>
-      <c r="F24" s="196">
-        <f>E24*C24</f>
-        <v/>
+      <c r="F24" s="196" t="n">
+        <v>400</v>
       </c>
       <c r="G24" s="140" t="n"/>
       <c r="H24" s="140" t="n"/>
@@ -2650,9 +2624,8 @@
       <c r="E25" s="189" t="n">
         <v>700</v>
       </c>
-      <c r="F25" s="189">
-        <f>E25*C25</f>
-        <v/>
+      <c r="F25" s="189" t="n">
+        <v>700</v>
       </c>
       <c r="G25" s="140" t="n"/>
       <c r="H25" s="140" t="n"/>
@@ -2692,9 +2665,8 @@
       <c r="E26" s="196" t="n">
         <v>47</v>
       </c>
-      <c r="F26" s="196">
-        <f>E26*C26</f>
-        <v/>
+      <c r="F26" s="196" t="n">
+        <v>0</v>
       </c>
       <c r="G26" s="140" t="n"/>
       <c r="H26" s="140" t="n"/>
@@ -2731,13 +2703,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="E27" s="189">
-        <f>SUM(F21:F26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="189">
-        <f>E27*C27/100</f>
-        <v/>
+      <c r="E27" s="189" t="n">
+        <v>43199.69</v>
+      </c>
+      <c r="F27" s="189" t="n">
+        <v>0</v>
       </c>
       <c r="G27" s="140" t="n"/>
       <c r="H27" s="140" t="n"/>
@@ -2769,9 +2739,8 @@
       <c r="C28" s="218" t="n"/>
       <c r="D28" s="218" t="n"/>
       <c r="E28" s="218" t="n"/>
-      <c r="F28" s="219">
-        <f>SUM(F22:F27)</f>
-        <v/>
+      <c r="F28" s="219" t="n">
+        <v>2207.93</v>
       </c>
       <c r="G28" s="140" t="n"/>
       <c r="H28" s="140" t="n"/>
@@ -2808,13 +2777,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="E29" s="189">
-        <f>SUM(F21:F27)</f>
-        <v/>
-      </c>
-      <c r="F29" s="189">
-        <f>E29*C29/100</f>
-        <v/>
+      <c r="E29" s="189" t="n">
+        <v>43199.69</v>
+      </c>
+      <c r="F29" s="189" t="n">
+        <v>1943.99</v>
       </c>
       <c r="G29" s="140" t="n"/>
       <c r="H29" s="140" t="n"/>
@@ -2854,9 +2821,8 @@
       <c r="E30" s="196" t="n">
         <v>36</v>
       </c>
-      <c r="F30" s="196">
-        <f>E30*C30</f>
-        <v/>
+      <c r="F30" s="196" t="n">
+        <v>-900</v>
       </c>
       <c r="G30" s="140" t="n"/>
       <c r="H30" s="140" t="n"/>
@@ -2896,9 +2862,8 @@
       <c r="E31" s="189" t="n">
         <v>43</v>
       </c>
-      <c r="F31" s="189">
-        <f>E31*C31</f>
-        <v/>
+      <c r="F31" s="189" t="n">
+        <v>-860</v>
       </c>
       <c r="G31" s="140" t="n"/>
       <c r="H31" s="140" t="n"/>
@@ -2973,9 +2938,8 @@
       <c r="C33" s="205" t="n"/>
       <c r="D33" s="205" t="n"/>
       <c r="E33" s="205" t="n"/>
-      <c r="F33" s="206">
-        <f>F28+I15+F32</f>
-        <v/>
+      <c r="F33" s="206" t="n">
+        <v>43699.69</v>
       </c>
       <c r="G33" s="140" t="n"/>
       <c r="H33" s="140" t="n"/>
@@ -3040,9 +3004,8 @@
       <c r="C35" s="205" t="n"/>
       <c r="D35" s="205" t="n"/>
       <c r="E35" s="205" t="n"/>
-      <c r="F35" s="206">
-        <f>F34-F33</f>
-        <v/>
+      <c r="F35" s="206" t="n">
+        <v>2500.31</v>
       </c>
       <c r="G35" s="143" t="n"/>
       <c r="H35" s="143" t="n"/>
@@ -3201,24 +3164,20 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D7" s="189">
-        <f>Raipur!E7+3100</f>
-        <v/>
-      </c>
-      <c r="E7" s="189">
-        <f>D7*B7/100</f>
-        <v/>
+      <c r="D7" s="189" t="n">
+        <v>29400</v>
+      </c>
+      <c r="E7" s="189" t="n">
+        <v>11172</v>
       </c>
       <c r="F7" s="190" t="n">
         <v>0.79</v>
       </c>
-      <c r="G7" s="189">
-        <f>E7/F7</f>
-        <v/>
-      </c>
-      <c r="H7" s="189">
-        <f>G7</f>
-        <v/>
+      <c r="G7" s="189" t="n">
+        <v>14141.77</v>
+      </c>
+      <c r="H7" s="189" t="n">
+        <v>14141.77</v>
       </c>
     </row>
     <row r="8">
@@ -3235,24 +3194,20 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D8" s="196">
-        <f>Raipur!E8+3100</f>
-        <v/>
-      </c>
-      <c r="E8" s="196">
-        <f>D8*B8/100</f>
-        <v/>
+      <c r="D8" s="196" t="n">
+        <v>40400</v>
+      </c>
+      <c r="E8" s="196" t="n">
+        <v>4848</v>
       </c>
       <c r="F8" s="197" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="G8" s="196">
-        <f>E8/F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="196">
-        <f>G8</f>
-        <v/>
+      <c r="G8" s="196" t="n">
+        <v>5157.45</v>
+      </c>
+      <c r="H8" s="196" t="n">
+        <v>5157.45</v>
       </c>
     </row>
     <row r="9">
@@ -3269,24 +3224,20 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D9" s="188">
-        <f>35500-500</f>
-        <v/>
-      </c>
-      <c r="E9" s="189">
-        <f>D9*B9/100</f>
-        <v/>
+      <c r="D9" s="188" t="n">
+        <v>35000</v>
+      </c>
+      <c r="E9" s="189" t="n">
+        <v>17500</v>
       </c>
       <c r="F9" s="190" t="n">
         <v>0.96</v>
       </c>
-      <c r="G9" s="189">
-        <f>E9/F9</f>
-        <v/>
-      </c>
-      <c r="H9" s="189">
-        <f>G9</f>
-        <v/>
+      <c r="G9" s="189" t="n">
+        <v>18229.17</v>
+      </c>
+      <c r="H9" s="189" t="n">
+        <v>18229.17</v>
       </c>
     </row>
     <row r="10">
@@ -3303,24 +3254,20 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D10" s="196">
-        <f>Raipur!E10</f>
-        <v/>
-      </c>
-      <c r="E10" s="196">
-        <f>D10*B10</f>
-        <v/>
+      <c r="D10" s="196" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="E10" s="196" t="n">
+        <v>1044.4</v>
       </c>
       <c r="F10" s="197" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="196">
-        <f>E10/F10</f>
-        <v/>
-      </c>
-      <c r="H10" s="196">
-        <f>G10</f>
-        <v/>
+      <c r="G10" s="196" t="n">
+        <v>1044.4</v>
+      </c>
+      <c r="H10" s="196" t="n">
+        <v>1044.4</v>
       </c>
     </row>
     <row r="11">
@@ -3337,24 +3284,20 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D11" s="189">
-        <f>Raipur!E11+3100</f>
-        <v/>
-      </c>
-      <c r="E11" s="189">
-        <f>D11*B11/100</f>
-        <v/>
+      <c r="D11" s="189" t="n">
+        <v>33300</v>
+      </c>
+      <c r="E11" s="189" t="n">
+        <v>0</v>
       </c>
       <c r="F11" s="190" t="n">
         <v>0.83</v>
       </c>
-      <c r="G11" s="189">
-        <f>E11/F11</f>
-        <v/>
-      </c>
-      <c r="H11" s="189">
-        <f>G11</f>
-        <v/>
+      <c r="G11" s="189" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="189" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -3370,15 +3313,13 @@
       <c r="D12" s="196" t="n">
         <v>6.5</v>
       </c>
-      <c r="E12" s="196">
-        <f>D12*B12</f>
-        <v/>
+      <c r="E12" s="196" t="n">
+        <v>4225</v>
       </c>
       <c r="F12" s="197" t="n"/>
       <c r="G12" s="200" t="n"/>
-      <c r="H12" s="196">
-        <f>D12*B12</f>
-        <v/>
+      <c r="H12" s="196" t="n">
+        <v>4225</v>
       </c>
     </row>
     <row r="13">
@@ -3398,15 +3339,13 @@
       <c r="D13" s="189" t="n">
         <v>500</v>
       </c>
-      <c r="E13" s="189">
-        <f>D13*B13</f>
-        <v/>
+      <c r="E13" s="189" t="n">
+        <v>500</v>
       </c>
       <c r="F13" s="190" t="n"/>
       <c r="G13" s="202" t="n"/>
-      <c r="H13" s="189">
-        <f>D13*B13</f>
-        <v/>
+      <c r="H13" s="189" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="14">
@@ -3426,15 +3365,13 @@
       <c r="D14" s="196" t="n">
         <v>550</v>
       </c>
-      <c r="E14" s="196">
-        <f>D14</f>
-        <v/>
+      <c r="E14" s="196" t="n">
+        <v>550</v>
       </c>
       <c r="F14" s="197" t="n"/>
       <c r="G14" s="200" t="n"/>
-      <c r="H14" s="196">
-        <f>D14*B14</f>
-        <v/>
+      <c r="H14" s="196" t="n">
+        <v>550</v>
       </c>
     </row>
     <row r="15">
@@ -3443,21 +3380,20 @@
           <t>Billet Cost</t>
         </is>
       </c>
-      <c r="B15" s="205">
-        <f>Raipur!B15</f>
-        <v/>
-      </c>
-      <c r="C15" s="204">
-        <f>Raipur!C15</f>
-        <v/>
+      <c r="B15" s="205" t="inlineStr">
+        <is>
+          <t>Billet Cost</t>
+        </is>
+      </c>
+      <c r="C15" s="204" t="n">
+        <v>46104</v>
       </c>
       <c r="D15" s="205" t="n"/>
       <c r="E15" s="205" t="n"/>
       <c r="F15" s="205" t="n"/>
       <c r="G15" s="205" t="n"/>
-      <c r="H15" s="206">
-        <f>SUM(H7:H14)</f>
-        <v/>
+      <c r="H15" s="206" t="n">
+        <v>43847.79</v>
       </c>
     </row>
     <row r="16">
@@ -3476,9 +3412,8 @@
       <c r="E16" s="209" t="n"/>
       <c r="F16" s="209" t="n"/>
       <c r="G16" s="209" t="n"/>
-      <c r="H16" s="188">
-        <f>44300-500</f>
-        <v/>
+      <c r="H16" s="188" t="n">
+        <v>43800</v>
       </c>
     </row>
     <row r="17">
@@ -3497,9 +3432,8 @@
       <c r="E17" s="205" t="n"/>
       <c r="F17" s="205" t="n"/>
       <c r="G17" s="205" t="n"/>
-      <c r="H17" s="206">
-        <f>H16-H15</f>
-        <v/>
+      <c r="H17" s="206" t="n">
+        <v>-47.79</v>
       </c>
     </row>
     <row r="18">
@@ -3582,9 +3516,8 @@
       <c r="C21" s="202" t="n"/>
       <c r="D21" s="202" t="n"/>
       <c r="E21" s="202" t="n"/>
-      <c r="F21" s="189">
-        <f>H15</f>
-        <v/>
+      <c r="F21" s="189" t="n">
+        <v>43847.79</v>
       </c>
       <c r="G21" s="141" t="n"/>
       <c r="H21" s="141" t="n"/>
@@ -3608,13 +3541,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="E22" s="196">
-        <f>H15</f>
-        <v/>
-      </c>
-      <c r="F22" s="196">
-        <f>E22*C22/100</f>
-        <v/>
+      <c r="E22" s="196" t="n">
+        <v>43847.79</v>
+      </c>
+      <c r="F22" s="196" t="n">
+        <v>350.78</v>
       </c>
       <c r="G22" s="140" t="n"/>
       <c r="H22" s="140" t="n"/>
@@ -3641,9 +3572,8 @@
       <c r="E23" s="189" t="n">
         <v>6.5</v>
       </c>
-      <c r="F23" s="189">
-        <f>E23*C23</f>
-        <v/>
+      <c r="F23" s="189" t="n">
+        <v>780</v>
       </c>
       <c r="G23" s="140" t="n"/>
       <c r="H23" s="140" t="n"/>
@@ -3670,9 +3600,8 @@
       <c r="E24" s="196" t="n">
         <v>400</v>
       </c>
-      <c r="F24" s="196">
-        <f>E24*C24</f>
-        <v/>
+      <c r="F24" s="196" t="n">
+        <v>400</v>
       </c>
       <c r="G24" s="140" t="n"/>
       <c r="H24" s="140" t="n"/>
@@ -3699,9 +3628,8 @@
       <c r="E25" s="189" t="n">
         <v>700</v>
       </c>
-      <c r="F25" s="189">
-        <f>E25*C25</f>
-        <v/>
+      <c r="F25" s="189" t="n">
+        <v>700</v>
       </c>
       <c r="G25" s="140" t="n"/>
       <c r="H25" s="140" t="n"/>
@@ -3728,9 +3656,8 @@
       <c r="E26" s="196" t="n">
         <v>47</v>
       </c>
-      <c r="F26" s="196">
-        <f>E26*C26</f>
-        <v/>
+      <c r="F26" s="196" t="n">
+        <v>0</v>
       </c>
       <c r="G26" s="140" t="n"/>
       <c r="H26" s="140" t="n"/>
@@ -3754,13 +3681,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="E27" s="189">
-        <f>SUM(F21:F26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="189">
-        <f>E27*C27/100</f>
-        <v/>
+      <c r="E27" s="189" t="n">
+        <v>46078.57</v>
+      </c>
+      <c r="F27" s="189" t="n">
+        <v>0</v>
       </c>
       <c r="G27" s="140" t="n"/>
       <c r="H27" s="140" t="n"/>
@@ -3779,9 +3704,8 @@
       <c r="C28" s="218" t="n"/>
       <c r="D28" s="218" t="n"/>
       <c r="E28" s="218" t="n"/>
-      <c r="F28" s="219">
-        <f>SUM(F22:F27)</f>
-        <v/>
+      <c r="F28" s="219" t="n">
+        <v>2230.78</v>
       </c>
       <c r="G28" s="140" t="n"/>
       <c r="H28" s="140" t="n"/>
@@ -3805,13 +3729,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="E29" s="189">
-        <f>SUM(F21:F27)</f>
-        <v/>
-      </c>
-      <c r="F29" s="189">
-        <f>E29*C29/100</f>
-        <v/>
+      <c r="E29" s="189" t="n">
+        <v>46078.57</v>
+      </c>
+      <c r="F29" s="189" t="n">
+        <v>2073.54</v>
       </c>
       <c r="G29" s="140" t="n"/>
       <c r="H29" s="140" t="n"/>
@@ -3838,9 +3760,8 @@
       <c r="E30" s="196" t="n">
         <v>36</v>
       </c>
-      <c r="F30" s="196">
-        <f>E30*C30</f>
-        <v/>
+      <c r="F30" s="196" t="n">
+        <v>-1620</v>
       </c>
       <c r="G30" s="140" t="n"/>
       <c r="H30" s="140" t="n"/>
@@ -3867,9 +3788,8 @@
       <c r="E31" s="189" t="n">
         <v>43</v>
       </c>
-      <c r="F31" s="189">
-        <f>E31*C31</f>
-        <v/>
+      <c r="F31" s="189" t="n">
+        <v>-860</v>
       </c>
       <c r="G31" s="140" t="n"/>
       <c r="H31" s="140" t="n"/>
@@ -3918,9 +3838,8 @@
       <c r="C33" s="205" t="n"/>
       <c r="D33" s="205" t="n"/>
       <c r="E33" s="205" t="n"/>
-      <c r="F33" s="206">
-        <f>H15+F28+F32</f>
-        <v/>
+      <c r="F33" s="206" t="n">
+        <v>46578.57</v>
       </c>
       <c r="G33" s="140" t="n"/>
       <c r="H33" s="140" t="n"/>
@@ -3959,9 +3878,8 @@
       <c r="C35" s="205" t="n"/>
       <c r="D35" s="205" t="n"/>
       <c r="E35" s="205" t="n"/>
-      <c r="F35" s="206">
-        <f>F34-F33</f>
-        <v/>
+      <c r="F35" s="206" t="n">
+        <v>4021.43</v>
       </c>
       <c r="G35" s="143" t="n"/>
       <c r="H35" s="143" t="n"/>

</xml_diff>

<commit_message>
Update costing output for 2026-03-23
</commit_message>
<xml_diff>
--- a/output/2026-03-23/20260323_Costing TMT.xlsx
+++ b/output/2026-03-23/20260323_Costing TMT.xlsx
@@ -1,20 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Raipur" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="NCR" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
+<s:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:workbookPr/>
+  <s:bookViews>
+    <s:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+  </s:bookViews>
+  <s:sheets>
+    <s:sheet name="Raipur" sheetId="1" state="visible" r:id="rId1"/>
+    <s:sheet name="NCR" sheetId="2" state="visible" r:id="rId2"/>
+  </s:sheets>
+  <s:definedNames/>
+  <s:calcPr calcId="191029" fullCalcOnLoad="1"/>
+</s:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1384,82 +1381,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Sumit K</author>
-  </authors>
-  <commentList>
-    <comment ref="B10" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Sumit K:
-25-150 mm, HC 60-14 
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Sumit K</author>
-  </authors>
-  <commentList>
-    <comment ref="A10" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Sumit K:
-25-150 mm, HC 60-14 
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
-    <sheetNames>
-      <sheetName val="Sheet1"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="Steel Mint Inputs"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="53">
-          <cell r="F53">
-            <v>41582.325872340429</v>
-          </cell>
-          <cell r="O53">
-            <v>44443.723852410454</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="F54">
-            <v>42000</v>
-          </cell>
-          <cell r="O54">
-            <v>45500</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="F55">
-            <v>417.67412765957124</v>
-          </cell>
-          <cell r="O55">
-            <v>1056.2761475895459</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>